<commit_message>
update on MSA; added dispersion in plots
</commit_message>
<xml_diff>
--- a/HazardAnalysis/gm-selection/2020_NBC_MyCopy_new-main/GMSelection_NGA_KiK_mixed/30GM_1p84_SF5_Guw_diffDeltaM.xlsx
+++ b/HazardAnalysis/gm-selection/2020_NBC_MyCopy_new-main/GMSelection_NGA_KiK_mixed/30GM_1p84_SF5_Guw_diffDeltaM.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52C912AD-16E7-48B2-BA05-4B97A44D987D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GMSel_ΔM (±)" sheetId="1" r:id="rId1"/>
@@ -1048,10 +1048,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="5" xfId="2" applyFont="1" applyAlignment="1">
@@ -27037,36 +27037,36 @@
       <c r="A2" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="43" t="s">
         <v>137</v>
       </c>
-      <c r="C2" s="43" t="s">
+      <c r="C2" s="44" t="s">
         <v>139</v>
       </c>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43" t="s">
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44" t="s">
         <v>161</v>
       </c>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
-      <c r="I2" s="43" t="s">
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44" t="s">
         <v>140</v>
       </c>
-      <c r="J2" s="43"/>
-      <c r="K2" s="43"/>
-      <c r="L2" s="43" t="s">
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44" t="s">
         <v>162</v>
       </c>
-      <c r="M2" s="43"/>
-      <c r="N2" s="43"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
       <c r="O2" s="1"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
     <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="45"/>
-      <c r="B3" s="44"/>
+      <c r="B3" s="43"/>
       <c r="C3" s="38" t="s">
         <v>109</v>
       </c>
@@ -27108,7 +27108,7 @@
       <c r="Q3" s="1"/>
     </row>
     <row r="4" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="44" t="s">
+      <c r="A4" s="43" t="s">
         <v>138</v>
       </c>
       <c r="C4" s="1">
@@ -27153,7 +27153,7 @@
       </c>
     </row>
     <row r="5" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="44"/>
+      <c r="A5" s="43"/>
       <c r="C5" s="1">
         <v>0.49</v>
       </c>
@@ -27211,7 +27211,7 @@
       <c r="Q6" s="1"/>
     </row>
     <row r="7" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A7" s="44" t="s">
+      <c r="A7" s="43" t="s">
         <v>160</v>
       </c>
       <c r="B7" s="39"/>
@@ -27257,7 +27257,7 @@
       </c>
     </row>
     <row r="8" spans="1:30" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="44"/>
+      <c r="A8" s="43"/>
       <c r="B8" s="39"/>
       <c r="C8" s="1">
         <v>0.46</v>
@@ -27328,33 +27328,33 @@
       <c r="A14" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="B14" s="44" t="s">
+      <c r="B14" s="43" t="s">
         <v>171</v>
       </c>
-      <c r="C14" s="43" t="s">
+      <c r="C14" s="44" t="s">
         <v>141</v>
       </c>
-      <c r="D14" s="43"/>
-      <c r="E14" s="43"/>
-      <c r="F14" s="43" t="s">
+      <c r="D14" s="44"/>
+      <c r="E14" s="44"/>
+      <c r="F14" s="44" t="s">
         <v>142</v>
       </c>
-      <c r="G14" s="43"/>
-      <c r="H14" s="43"/>
-      <c r="I14" s="43" t="s">
+      <c r="G14" s="44"/>
+      <c r="H14" s="44"/>
+      <c r="I14" s="44" t="s">
         <v>139</v>
       </c>
-      <c r="J14" s="43"/>
-      <c r="K14" s="43"/>
-      <c r="L14" s="43" t="s">
+      <c r="J14" s="44"/>
+      <c r="K14" s="44"/>
+      <c r="L14" s="44" t="s">
         <v>159</v>
       </c>
-      <c r="M14" s="43"/>
-      <c r="N14" s="43"/>
+      <c r="M14" s="44"/>
+      <c r="N14" s="44"/>
     </row>
     <row r="15" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="45"/>
-      <c r="B15" s="44"/>
+      <c r="B15" s="43"/>
       <c r="C15" s="38" t="s">
         <v>109</v>
       </c>
@@ -27393,7 +27393,7 @@
       </c>
     </row>
     <row r="16" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A16" s="44" t="s">
+      <c r="A16" s="43" t="s">
         <v>138</v>
       </c>
       <c r="C16" s="1">
@@ -27438,7 +27438,7 @@
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="44"/>
+      <c r="A17" s="43"/>
       <c r="C17" s="1">
         <v>0.46</v>
       </c>
@@ -27496,7 +27496,7 @@
       <c r="N18" s="23"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="44" t="s">
+      <c r="A19" s="43" t="s">
         <v>160</v>
       </c>
       <c r="B19" s="39"/>
@@ -27542,7 +27542,7 @@
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="44"/>
+      <c r="A20" s="43"/>
       <c r="B20" s="39"/>
       <c r="C20" s="1">
         <v>0.48</v>
@@ -27602,33 +27602,33 @@
       <c r="A27" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="B27" s="44" t="s">
+      <c r="B27" s="43" t="s">
         <v>172</v>
       </c>
-      <c r="C27" s="43" t="s">
+      <c r="C27" s="44" t="s">
         <v>163</v>
       </c>
-      <c r="D27" s="43"/>
-      <c r="E27" s="43"/>
-      <c r="F27" s="43" t="s">
+      <c r="D27" s="44"/>
+      <c r="E27" s="44"/>
+      <c r="F27" s="44" t="s">
         <v>164</v>
       </c>
-      <c r="G27" s="43"/>
-      <c r="H27" s="43"/>
-      <c r="I27" s="43" t="s">
+      <c r="G27" s="44"/>
+      <c r="H27" s="44"/>
+      <c r="I27" s="44" t="s">
         <v>165</v>
       </c>
-      <c r="J27" s="43"/>
-      <c r="K27" s="43"/>
-      <c r="L27" s="43" t="s">
+      <c r="J27" s="44"/>
+      <c r="K27" s="44"/>
+      <c r="L27" s="44" t="s">
         <v>166</v>
       </c>
-      <c r="M27" s="43"/>
-      <c r="N27" s="43"/>
+      <c r="M27" s="44"/>
+      <c r="N27" s="44"/>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="45"/>
-      <c r="B28" s="44"/>
+      <c r="B28" s="43"/>
       <c r="C28" s="38" t="s">
         <v>109</v>
       </c>
@@ -27667,7 +27667,7 @@
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="44" t="s">
+      <c r="A29" s="43" t="s">
         <v>138</v>
       </c>
       <c r="C29" s="1">
@@ -27712,7 +27712,7 @@
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="44"/>
+      <c r="A30" s="43"/>
       <c r="C30" s="1">
         <v>0.4</v>
       </c>
@@ -27770,7 +27770,7 @@
       <c r="N31" s="1"/>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A32" s="44" t="s">
+      <c r="A32" s="43" t="s">
         <v>160</v>
       </c>
       <c r="B32" s="39"/>
@@ -27816,7 +27816,7 @@
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A33" s="44"/>
+      <c r="A33" s="43"/>
       <c r="B33" s="39"/>
       <c r="C33" s="1">
         <v>0.37</v>
@@ -27903,16 +27903,12 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="I2:K2"/>
-    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="F14:H14"/>
+    <mergeCell ref="I14:K14"/>
+    <mergeCell ref="I27:K27"/>
+    <mergeCell ref="L27:N27"/>
+    <mergeCell ref="L14:N14"/>
+    <mergeCell ref="F27:H27"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="A7:A8"/>
     <mergeCell ref="A2:A3"/>
@@ -27920,13 +27916,17 @@
     <mergeCell ref="A27:A28"/>
     <mergeCell ref="A16:A17"/>
     <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:E27"/>
     <mergeCell ref="C14:E14"/>
-    <mergeCell ref="F14:H14"/>
-    <mergeCell ref="I14:K14"/>
-    <mergeCell ref="I27:K27"/>
-    <mergeCell ref="L27:N27"/>
-    <mergeCell ref="L14:N14"/>
-    <mergeCell ref="F27:H27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>